<commit_message>
Add accident archive reference feature and improve AI prompt work-name reflection
- Add cached loader and keyword-based search over the KOSHA high-risk accident
  archive, combined with the existing hazard_mapping DB as a second reference
  source for TBM hazard/measure generation (capped at top matches per source)
- Add an explicit work-name/work-content block at the top of the AI prompt so
  equipment-specific terms (e.g. pump, valve, welding) are reliably reflected
  in generated risk items and safety measures
- Tighten TBM history list row spacing (CSS)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hazard_mapping.xlsx
+++ b/hazard_mapping.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\화학시설검사부\경영평가\화학안전신호등\data_setup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\화학시설검사부\경영평가\화학안전신호등\data_setup\최신data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48624DAA-A9AF-41D4-B2F8-332D8A12CAAC}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{285672E7-623B-46D2-BE0B-E91FB0833A19}" xr6:coauthVersionLast="37" xr6:coauthVersionMax="37" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17250" windowHeight="5085" xr2:uid="{FBAE53C3-CE8F-41FC-8E58-FCC920D6A424}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$1:$D$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$F$95</definedName>
   </definedNames>
   <calcPr calcId="179021"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="126">
   <si>
     <t>연번</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -463,6 +463,21 @@
   <si>
     <t>물질군</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>특정표적장기 독성(2회 노출)</t>
+  </si>
+  <si>
+    <t>특정표적장기 독성(3회 노출)</t>
+  </si>
+  <si>
+    <t>특정표적장기 독성(4회 노출)</t>
+  </si>
+  <si>
+    <t>환경으로 배출 금지, 누출물 회수 및 유출 확산 방지, 우수로·배수구 유입 차단, 방유제·받침대 등 3차 containment 확보, 폐기물은 관련 법령에 따라 처리</t>
+  </si>
+  <si>
+    <t>환경으로 배출 금지, 누출물 회수 및 유출 확산 방지, 우수로·배수구 유입 차단, 방유제·받침대 등 4차 containment 확보, 폐기물은 관련 법령에 따라 처리</t>
   </si>
 </sst>
 </file>
@@ -826,9 +841,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB2C7B42-E318-4E4F-B3C7-D6BB75FC2E35}">
-  <dimension ref="A1:H90"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="11.875" customWidth="1"/>
     <col min="3" max="3" width="19.625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1280,6 +1296,9 @@
       <c r="A19">
         <v>18</v>
       </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
       <c r="C19" t="s">
         <v>36</v>
       </c>
@@ -1303,6 +1322,9 @@
       <c r="A20">
         <v>19</v>
       </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
       <c r="C20" t="s">
         <v>49</v>
       </c>
@@ -1340,6 +1362,9 @@
       <c r="A22">
         <v>21</v>
       </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
       <c r="C22" t="s">
         <v>48</v>
       </c>
@@ -1351,6 +1376,9 @@
       <c r="A23">
         <v>22</v>
       </c>
+      <c r="B23" t="s">
+        <v>8</v>
+      </c>
       <c r="C23" t="s">
         <v>37</v>
       </c>
@@ -1362,6 +1390,9 @@
       <c r="A24">
         <v>23</v>
       </c>
+      <c r="B24" t="s">
+        <v>8</v>
+      </c>
       <c r="C24" t="s">
         <v>50</v>
       </c>
@@ -1399,6 +1430,9 @@
       <c r="A26">
         <v>25</v>
       </c>
+      <c r="B26" t="s">
+        <v>121</v>
+      </c>
       <c r="C26" t="s">
         <v>37</v>
       </c>
@@ -1422,6 +1456,9 @@
       <c r="A27">
         <v>26</v>
       </c>
+      <c r="B27" t="s">
+        <v>122</v>
+      </c>
       <c r="C27" t="s">
         <v>51</v>
       </c>
@@ -1445,6 +1482,9 @@
       <c r="A28">
         <v>27</v>
       </c>
+      <c r="B28" t="s">
+        <v>123</v>
+      </c>
       <c r="C28" t="s">
         <v>52</v>
       </c>
@@ -1482,6 +1522,9 @@
       <c r="A30">
         <v>29</v>
       </c>
+      <c r="B30" t="s">
+        <v>10</v>
+      </c>
       <c r="C30" t="s">
         <v>37</v>
       </c>
@@ -1507,6 +1550,9 @@
       <c r="A32">
         <v>31</v>
       </c>
+      <c r="B32" t="s">
+        <v>11</v>
+      </c>
       <c r="C32" t="s">
         <v>37</v>
       </c>
@@ -1544,6 +1590,9 @@
       <c r="A34">
         <v>33</v>
       </c>
+      <c r="B34" t="s">
+        <v>12</v>
+      </c>
       <c r="C34" t="s">
         <v>37</v>
       </c>
@@ -1567,6 +1616,9 @@
       <c r="A35">
         <v>34</v>
       </c>
+      <c r="B35" t="s">
+        <v>12</v>
+      </c>
       <c r="C35" t="s">
         <v>53</v>
       </c>
@@ -1616,6 +1668,9 @@
       <c r="A37">
         <v>36</v>
       </c>
+      <c r="B37" t="s">
+        <v>13</v>
+      </c>
       <c r="C37" t="s">
         <v>55</v>
       </c>
@@ -1653,6 +1708,9 @@
       <c r="A39">
         <v>38</v>
       </c>
+      <c r="B39" t="s">
+        <v>14</v>
+      </c>
       <c r="C39" t="s">
         <v>36</v>
       </c>
@@ -1664,6 +1722,9 @@
       <c r="A40">
         <v>39</v>
       </c>
+      <c r="B40" t="s">
+        <v>14</v>
+      </c>
       <c r="C40" t="s">
         <v>49</v>
       </c>
@@ -1675,6 +1736,9 @@
       <c r="A41">
         <v>40</v>
       </c>
+      <c r="B41" t="s">
+        <v>14</v>
+      </c>
       <c r="C41" t="s">
         <v>58</v>
       </c>
@@ -1700,6 +1764,9 @@
       <c r="A43">
         <v>42</v>
       </c>
+      <c r="B43" t="s">
+        <v>15</v>
+      </c>
       <c r="C43" t="s">
         <v>36</v>
       </c>
@@ -1738,46 +1805,79 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C45" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="D45" t="s">
-        <v>56</v>
+        <v>36</v>
+      </c>
+      <c r="E45">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s">
+        <v>16</v>
+      </c>
+      <c r="G45" t="s">
+        <v>104</v>
+      </c>
+      <c r="H45" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
+      <c r="B46" t="s">
+        <v>16</v>
+      </c>
       <c r="C46" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="D46" t="s">
-        <v>36</v>
+        <v>49</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46" t="s">
+        <v>16</v>
+      </c>
+      <c r="G46" t="s">
+        <v>104</v>
+      </c>
+      <c r="H46" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
+      <c r="B47" t="s">
+        <v>17</v>
+      </c>
       <c r="C47" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D47" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
+      <c r="B48" t="s">
+        <v>17</v>
+      </c>
       <c r="C48" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="D48" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
@@ -1785,25 +1885,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C49" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D49" t="s">
-        <v>56</v>
-      </c>
-      <c r="E49">
-        <v>3</v>
-      </c>
-      <c r="F49" t="s">
-        <v>71</v>
-      </c>
-      <c r="G49" t="s">
-        <v>89</v>
-      </c>
-      <c r="H49" t="s">
-        <v>90</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
@@ -1811,58 +1899,91 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C50" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D50" t="s">
-        <v>56</v>
-      </c>
-      <c r="F50" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
+      <c r="B51" t="s">
+        <v>18</v>
+      </c>
       <c r="C51" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="D51" t="s">
-        <v>36</v>
+        <v>56</v>
+      </c>
+      <c r="E51">
+        <v>3</v>
       </c>
       <c r="F51" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+      <c r="G51" t="s">
+        <v>89</v>
+      </c>
+      <c r="H51" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
+      <c r="B52" t="s">
+        <v>18</v>
+      </c>
       <c r="C52" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="D52" t="s">
-        <v>49</v>
+        <v>36</v>
+      </c>
+      <c r="E52">
+        <v>2</v>
       </c>
       <c r="F52" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+      <c r="G52" t="s">
+        <v>89</v>
+      </c>
+      <c r="H52" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
+      <c r="B53" t="s">
+        <v>18</v>
+      </c>
       <c r="C53" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="D53" t="s">
-        <v>58</v>
+        <v>49</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
       </c>
       <c r="F53" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+      <c r="G53" t="s">
+        <v>89</v>
+      </c>
+      <c r="H53" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
@@ -1870,48 +1991,27 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C54" t="s">
         <v>57</v>
       </c>
       <c r="D54" t="s">
         <v>56</v>
-      </c>
-      <c r="E54">
-        <v>3</v>
-      </c>
-      <c r="F54" t="s">
-        <v>72</v>
-      </c>
-      <c r="G54" t="s">
-        <v>93</v>
-      </c>
-      <c r="H54" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
+      <c r="B55" t="s">
+        <v>19</v>
+      </c>
       <c r="C55" t="s">
         <v>36</v>
       </c>
       <c r="D55" t="s">
         <v>36</v>
-      </c>
-      <c r="E55">
-        <v>2</v>
-      </c>
-      <c r="F55" t="s">
-        <v>72</v>
-      </c>
-      <c r="G55" t="s">
-        <v>93</v>
-      </c>
-      <c r="H55" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
@@ -1919,94 +2019,79 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C56" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D56" t="s">
-        <v>56</v>
-      </c>
-      <c r="E56">
-        <v>3</v>
-      </c>
-      <c r="F56" t="s">
-        <v>69</v>
-      </c>
-      <c r="G56" t="s">
-        <v>81</v>
-      </c>
-      <c r="H56" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
+      <c r="B57" t="s">
+        <v>19</v>
+      </c>
       <c r="C57" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="D57" t="s">
-        <v>36</v>
-      </c>
-      <c r="E57">
-        <v>2</v>
-      </c>
-      <c r="F57" t="s">
-        <v>69</v>
-      </c>
-      <c r="G57" t="s">
-        <v>81</v>
-      </c>
-      <c r="H57" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
+      <c r="B58" t="s">
+        <v>20</v>
+      </c>
       <c r="C58" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D58" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F58" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G58" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="H58" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
+      <c r="B59" t="s">
+        <v>20</v>
+      </c>
       <c r="C59" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="D59" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="E59">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F59" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G59" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="H59" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.3">
@@ -2014,48 +2099,48 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C60" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D60" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F60" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G60" t="s">
-        <v>106</v>
-      </c>
-      <c r="H60" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
+      <c r="B61" t="s">
+        <v>21</v>
+      </c>
       <c r="C61" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D61" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G61" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="H61" t="s">
-        <v>107</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
@@ -2063,13 +2148,25 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C62" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="D62" t="s">
-        <v>56</v>
+        <v>36</v>
+      </c>
+      <c r="E62">
+        <v>2</v>
+      </c>
+      <c r="F62" t="s">
+        <v>69</v>
+      </c>
+      <c r="G62" t="s">
+        <v>81</v>
+      </c>
+      <c r="H62" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.3">
@@ -2077,59 +2174,65 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C63" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="D63" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E63">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F63" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G63" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="H63" t="s">
-        <v>109</v>
+        <v>82</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
+      <c r="B64" t="s">
+        <v>21</v>
+      </c>
       <c r="C64" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D64" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E64">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F64" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="G64" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="H64" t="s">
-        <v>109</v>
+        <v>82</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
+      <c r="B65" t="s">
+        <v>23</v>
+      </c>
       <c r="C65" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D65" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E65">
         <v>3</v>
@@ -2138,64 +2241,61 @@
         <v>74</v>
       </c>
       <c r="G65" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H65" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
+      <c r="B66" t="s">
+        <v>23</v>
+      </c>
       <c r="C66" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D66" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="E66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F66" t="s">
         <v>74</v>
       </c>
       <c r="G66" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H66" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
+      <c r="B67" t="s">
+        <v>24</v>
+      </c>
       <c r="C67" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="D67" t="s">
-        <v>57</v>
-      </c>
-      <c r="E67">
-        <v>3</v>
-      </c>
-      <c r="F67" t="s">
-        <v>74</v>
-      </c>
-      <c r="G67" t="s">
-        <v>108</v>
-      </c>
-      <c r="H67" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
+      <c r="B68" t="s">
+        <v>25</v>
+      </c>
       <c r="C68" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D68" t="s">
         <v>57</v>
@@ -2217,8 +2317,11 @@
       <c r="A69">
         <v>68</v>
       </c>
+      <c r="B69" t="s">
+        <v>25</v>
+      </c>
       <c r="C69" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D69" t="s">
         <v>57</v>
@@ -2241,35 +2344,77 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C70" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D70" t="s">
         <v>57</v>
+      </c>
+      <c r="E70">
+        <v>3</v>
+      </c>
+      <c r="F70" t="s">
+        <v>74</v>
+      </c>
+      <c r="G70" t="s">
+        <v>108</v>
+      </c>
+      <c r="H70" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
+      <c r="B71" t="s">
+        <v>25</v>
+      </c>
       <c r="C71" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D71" t="s">
-        <v>59</v>
+        <v>57</v>
+      </c>
+      <c r="E71">
+        <v>3</v>
+      </c>
+      <c r="F71" t="s">
+        <v>74</v>
+      </c>
+      <c r="G71" t="s">
+        <v>108</v>
+      </c>
+      <c r="H71" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
+      <c r="B72" t="s">
+        <v>25</v>
+      </c>
       <c r="C72" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="D72" t="s">
-        <v>75</v>
+        <v>57</v>
+      </c>
+      <c r="E72">
+        <v>3</v>
+      </c>
+      <c r="F72" t="s">
+        <v>74</v>
+      </c>
+      <c r="G72" t="s">
+        <v>108</v>
+      </c>
+      <c r="H72" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -2277,10 +2422,10 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C73" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D73" t="s">
         <v>57</v>
@@ -2292,18 +2437,21 @@
         <v>74</v>
       </c>
       <c r="G73" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H73" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
+      <c r="B74" t="s">
+        <v>25</v>
+      </c>
       <c r="C74" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D74" t="s">
         <v>57</v>
@@ -2315,87 +2463,63 @@
         <v>74</v>
       </c>
       <c r="G74" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H74" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
+      <c r="B75" t="s">
+        <v>26</v>
+      </c>
       <c r="C75" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D75" t="s">
         <v>57</v>
-      </c>
-      <c r="E75">
-        <v>3</v>
-      </c>
-      <c r="F75" t="s">
-        <v>74</v>
-      </c>
-      <c r="G75" t="s">
-        <v>110</v>
-      </c>
-      <c r="H75" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
+      <c r="B76" t="s">
+        <v>26</v>
+      </c>
       <c r="C76" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D76" t="s">
-        <v>57</v>
-      </c>
-      <c r="E76">
-        <v>3</v>
-      </c>
-      <c r="F76" t="s">
-        <v>74</v>
-      </c>
-      <c r="G76" t="s">
-        <v>110</v>
-      </c>
-      <c r="H76" t="s">
-        <v>111</v>
+        <v>59</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
+      <c r="B77" t="s">
+        <v>26</v>
+      </c>
       <c r="C77" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D77" t="s">
-        <v>57</v>
-      </c>
-      <c r="E77">
-        <v>3</v>
-      </c>
-      <c r="F77" t="s">
-        <v>74</v>
-      </c>
-      <c r="G77" t="s">
-        <v>110</v>
-      </c>
-      <c r="H77" t="s">
-        <v>111</v>
+        <v>75</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
+      <c r="B78" t="s">
+        <v>27</v>
+      </c>
       <c r="C78" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D78" t="s">
         <v>57</v>
@@ -2417,8 +2541,11 @@
       <c r="A79">
         <v>78</v>
       </c>
+      <c r="B79" t="s">
+        <v>27</v>
+      </c>
       <c r="C79" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D79" t="s">
         <v>57</v>
@@ -2441,71 +2568,77 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C80" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D80" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E80">
         <v>3</v>
       </c>
       <c r="F80" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G80" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="H80" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
+      <c r="B81" t="s">
+        <v>27</v>
+      </c>
       <c r="C81" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D81" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="E81">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F81" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G81" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="H81" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
+      <c r="B82" t="s">
+        <v>27</v>
+      </c>
       <c r="C82" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="D82" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E82">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F82" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G82" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="H82" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.3">
@@ -2513,13 +2646,25 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C83" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="D83" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="E83">
+        <v>3</v>
+      </c>
+      <c r="F83" t="s">
+        <v>74</v>
+      </c>
+      <c r="G83" t="s">
+        <v>110</v>
+      </c>
+      <c r="H83" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.3">
@@ -2527,13 +2672,13 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C84" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D84" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E84">
         <v>3</v>
@@ -2542,10 +2687,10 @@
         <v>74</v>
       </c>
       <c r="G84" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H84" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.3">
@@ -2553,7 +2698,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C85" t="s">
         <v>57</v>
@@ -2565,19 +2710,22 @@
         <v>3</v>
       </c>
       <c r="F85" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G85" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H85" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
+      <c r="B86" t="s">
+        <v>28</v>
+      </c>
       <c r="C86" t="s">
         <v>36</v>
       </c>
@@ -2588,19 +2736,22 @@
         <v>2</v>
       </c>
       <c r="F86" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G86" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H86" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
+      <c r="B87" t="s">
+        <v>28</v>
+      </c>
       <c r="C87" t="s">
         <v>49</v>
       </c>
@@ -2611,13 +2762,13 @@
         <v>1</v>
       </c>
       <c r="F87" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G87" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H87" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.3">
@@ -2625,25 +2776,13 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C88" t="s">
         <v>57</v>
       </c>
       <c r="D88" t="s">
         <v>56</v>
-      </c>
-      <c r="E88">
-        <v>3</v>
-      </c>
-      <c r="F88" t="s">
-        <v>74</v>
-      </c>
-      <c r="G88" t="s">
-        <v>114</v>
-      </c>
-      <c r="H88" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.3">
@@ -2651,7 +2790,7 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C89" t="s">
         <v>57</v>
@@ -2666,10 +2805,10 @@
         <v>74</v>
       </c>
       <c r="G89" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H89" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.3">
@@ -2677,7 +2816,7 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C90" t="s">
         <v>57</v>
@@ -2689,17 +2828,147 @@
         <v>3</v>
       </c>
       <c r="F90" t="s">
+        <v>71</v>
+      </c>
+      <c r="G90" t="s">
+        <v>87</v>
+      </c>
+      <c r="H90" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>31</v>
+      </c>
+      <c r="C91" t="s">
+        <v>36</v>
+      </c>
+      <c r="D91" t="s">
+        <v>36</v>
+      </c>
+      <c r="E91">
+        <v>2</v>
+      </c>
+      <c r="F91" t="s">
+        <v>71</v>
+      </c>
+      <c r="G91" t="s">
+        <v>87</v>
+      </c>
+      <c r="H91" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>31</v>
+      </c>
+      <c r="C92" t="s">
+        <v>49</v>
+      </c>
+      <c r="D92" t="s">
+        <v>49</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+      <c r="F92" t="s">
+        <v>71</v>
+      </c>
+      <c r="G92" t="s">
+        <v>87</v>
+      </c>
+      <c r="H92" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>32</v>
+      </c>
+      <c r="C93" t="s">
+        <v>57</v>
+      </c>
+      <c r="D93" t="s">
+        <v>56</v>
+      </c>
+      <c r="E93">
+        <v>3</v>
+      </c>
+      <c r="F93" t="s">
         <v>74</v>
       </c>
-      <c r="G90" t="s">
+      <c r="G93" t="s">
+        <v>114</v>
+      </c>
+      <c r="H93" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>33</v>
+      </c>
+      <c r="C94" t="s">
+        <v>57</v>
+      </c>
+      <c r="D94" t="s">
+        <v>56</v>
+      </c>
+      <c r="E94">
+        <v>3</v>
+      </c>
+      <c r="F94" t="s">
+        <v>74</v>
+      </c>
+      <c r="G94" t="s">
+        <v>116</v>
+      </c>
+      <c r="H94" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>34</v>
+      </c>
+      <c r="C95" t="s">
+        <v>57</v>
+      </c>
+      <c r="D95" t="s">
+        <v>56</v>
+      </c>
+      <c r="E95">
+        <v>3</v>
+      </c>
+      <c r="F95" t="s">
+        <v>74</v>
+      </c>
+      <c r="G95" t="s">
         <v>118</v>
       </c>
-      <c r="H90" t="s">
+      <c r="H95" t="s">
         <v>119</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="D1:D90" xr:uid="{DA5BB3FD-1EB0-4AF9-98CF-93A43CE7645F}"/>
+  <autoFilter ref="B1:F95" xr:uid="{EF4B4680-52E5-4384-85A9-51601ED11A94}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>